<commit_message>
infor PeYa export v 1.1
</commit_message>
<xml_diff>
--- a/public/data/Infor00000.xlsx
+++ b/public/data/Infor00000.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JTOSO\Desktop\PeYa\Pedidos\Infor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JTOSO\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B7773FE3-57B6-4662-B941-FEA39961C6D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A7D8265-FF20-4AFA-877A-B7FEE60B85E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -40,420 +40,6 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>K France</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Do Not Change ROW 1.
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>These are database column names that must be present for import process</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Errors encountered during import will be logged in this column
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">For New orders you can either:
-</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>(a)</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve"> Leave the Order Number blank and use the generic key to let the system assign the order number.
-</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>(b)</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve"> leave the Generic Key blank and input desired Order Number</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">For New orders you can either:
-</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>(a)</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve"> Leave the Order Number blank and use the generic key to let the system assign the order number.
-</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>(b)</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve"> leave the Generic Key blank and input desired Order Number</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Required owner ID</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Define valid order types in the System Code ORDERTYPE</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>K France</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Do Not Change ROW 1.
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>These are database column names that must be present for import process</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Errors encountered during import will be logged in this column
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">For New orders you can either:
-</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>(a)</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve"> Leave the Order Number blank and use the generic key to let the system assign the order number.
-</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>(b)</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve"> leave the Generic Key blank and input desired Order Number</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">For New orders you can either:
-</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>(a)</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve"> Leave the Order Number blank and use the generic key to let the system assign the order number.
-</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>(b)</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve"> leave the Generic Key blank and input desired Order Number</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000005000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-REQUIRED</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G2" authorId="0" shapeId="0" xr:uid="{11836518-D101-4BDA-A814-15B0E14C7B32}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>IMPORT:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-This is the Order Quantity in  Master Units (Eaches)
-</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>EXPORT:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="8"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-This is the quantity (eaches) that has not been shipped</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="220">
   <si>
@@ -1121,7 +707,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1129,19 +715,6 @@
     <font>
       <sz val="8"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
     <font>
@@ -1302,25 +875,25 @@
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1624,7 +1197,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1705,12 +1278,11 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1950,7 +1522,6 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>